<commit_message>
Add inline GUI status checkmarks
</commit_message>
<xml_diff>
--- a/output/pony-cup_barn_schedule.xlsx
+++ b/output/pony-cup_barn_schedule.xlsx
@@ -13,13 +13,13 @@
     <sheet name="Sun" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Rides'!$A$3:$J$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Rides'!$A$3:$K$40</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'All Rides'!$1:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fri'!$A$3:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fri'!$A$3:$K$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Fri'!$1:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sat'!$A$3:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sat'!$A$3:$K$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Sat'!$1:$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sun'!$A$3:$J$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Sun'!$A$3:$K$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Sun'!$1:$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -462,11 +462,13 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -494,35 +496,40 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Rider</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Horse</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Class #</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Class Name</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Arena #</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Arena Name</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -540,37 +547,38 @@
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>1FI2EF</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediate II Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (J. Lees at C; C. Carlson at B)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -584,37 +592,38 @@
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>1PSG</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -628,37 +637,38 @@
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Destemido RRI</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -672,37 +682,38 @@
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -716,37 +727,38 @@
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>133</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -760,37 +772,38 @@
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>H1UB</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test B</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -804,37 +817,38 @@
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>121</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 1</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -848,37 +862,38 @@
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>1T3</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -892,37 +907,38 @@
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Edwards, Susan</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>JP Zeppelin</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>H122</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 2</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -936,37 +952,38 @@
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Sophie Bayer at C)</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -980,37 +997,38 @@
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Sophie Bayer at C)</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1024,37 +1042,38 @@
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>1FFS</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1068,37 +1087,38 @@
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>112</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>First Level Test 2</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>The Sanctuary (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1112,37 +1132,38 @@
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>1T3</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1156,37 +1177,38 @@
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 3</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1200,37 +1222,38 @@
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>Destemido RRI</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>H2PSG</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="J19" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1244,37 +1267,38 @@
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>H2I1</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="J20" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1288,37 +1312,38 @@
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Edwards, Susan</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>JP Zeppelin</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>H223</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 3</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="J21" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr"/>
+      <c r="K21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1332,37 +1357,38 @@
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr"/>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="J22" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1376,37 +1402,38 @@
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1420,37 +1447,38 @@
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr"/>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>H2UC</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test C</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="J24" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr"/>
+      <c r="K24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1464,37 +1492,38 @@
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="I25" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="J25" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr"/>
+      <c r="K25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1508,37 +1537,38 @@
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="J26" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr"/>
+      <c r="K26" s="4" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1552,37 +1582,38 @@
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>2T3</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="I27" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I27" s="3" t="inlineStr">
+      <c r="J27" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr"/>
+      <c r="K27" s="4" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1596,37 +1627,38 @@
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr"/>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="J28" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr"/>
+      <c r="K28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1640,37 +1672,38 @@
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="F29" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="J29" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr"/>
+      <c r="K29" s="4" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -1684,37 +1717,38 @@
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="J30" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr"/>
+      <c r="K30" s="4" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1728,37 +1762,38 @@
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>2I2</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare II</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
+      <c r="J31" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr"/>
+      <c r="K31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1772,37 +1807,38 @@
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr"/>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="F32" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>212</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>First Level Test 2</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="J32" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr"/>
+      <c r="K32" s="4" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1816,37 +1852,38 @@
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="F33" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>2YH</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="H33" s="3" t="inlineStr">
         <is>
           <t>Young Horse Test of Choice (excl 7YO)</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
+      <c r="I33" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I33" s="3" t="inlineStr">
+      <c r="J33" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr"/>
+      <c r="K33" s="4" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -1860,37 +1897,38 @@
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr"/>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr"/>
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>US4EF</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>USEF 4-Year-Old Test Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Beverly Rogers at C; Agnes</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr"/>
+      <c r="K34" s="4" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -1904,37 +1942,38 @@
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>DHGEF</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="H35" s="3" t="inlineStr">
         <is>
           <t>USEF Developing Horse Grand Prix Test Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I35" s="3" t="inlineStr">
+      <c r="J35" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr"/>
+      <c r="K35" s="4" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -1948,37 +1987,38 @@
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr"/>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
+      <c r="J36" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr"/>
+      <c r="K36" s="4" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -1992,37 +2032,38 @@
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>Edwards, Susan</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="F37" s="3" t="inlineStr">
         <is>
           <t>JP Zeppelin</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="G37" s="3" t="inlineStr">
         <is>
           <t>331</t>
         </is>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="H37" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 1</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="I37" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I37" s="3" t="inlineStr">
+      <c r="J37" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Cheryl Holekamp at C)</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr"/>
+      <c r="K37" s="4" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2036,37 +2077,38 @@
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr"/>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D38" s="4" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="G38" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr"/>
+      <c r="K38" s="4" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2080,37 +2122,38 @@
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr"/>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="F39" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="G39" s="3" t="inlineStr">
         <is>
           <t>3PSG</t>
         </is>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="H39" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I39" s="3" t="inlineStr">
+      <c r="J39" s="3" t="inlineStr">
         <is>
           <t>The Sanctuary (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr"/>
+      <c r="K39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2124,42 +2167,43 @@
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr"/>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D40" s="4" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="F40" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
+      <c r="G40" s="3" t="inlineStr">
         <is>
           <t>3FFS</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H40" s="3" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I40" s="3" t="inlineStr">
+      <c r="J40" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr"/>
+      <c r="K40" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J40"/>
+  <autoFilter ref="A3:K40"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2172,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2180,11 +2224,13 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2212,35 +2258,40 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Rider</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Horse</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Class #</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Class Name</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Arena #</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Arena Name</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -2258,37 +2309,38 @@
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>1FI2EF</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediate II Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (J. Lees at C; C. Carlson at B)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2302,37 +2354,38 @@
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>1PSG</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2346,37 +2399,38 @@
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Destemido RRI</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2390,37 +2444,38 @@
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>H1PSG</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>FEI Prix. St. Georges</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2434,37 +2489,38 @@
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>133</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2478,37 +2534,38 @@
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>H1UB</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test B</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2522,37 +2579,38 @@
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>121</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 1</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2566,37 +2624,38 @@
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>1T3</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2610,37 +2669,38 @@
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Edwards, Susan</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>JP Zeppelin</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>H122</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 2</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2654,37 +2714,38 @@
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Sophie Bayer at C)</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2698,37 +2759,38 @@
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>113</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Sophie Bayer at C)</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2742,37 +2804,38 @@
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>1FFS</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Beverly Rogers at C)</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2786,37 +2849,38 @@
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>112</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>First Level Test 2</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>The Sanctuary (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2830,37 +2894,38 @@
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>1T3</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2874,42 +2939,43 @@
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 3</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J18"/>
+  <autoFilter ref="A3:K18"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -2922,7 +2988,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2930,11 +2996,13 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2962,35 +3030,40 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Rider</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Horse</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Class #</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Class Name</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Arena #</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Arena Name</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3008,37 +3081,38 @@
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Destemido RRI</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>H2PSG</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3052,37 +3126,38 @@
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Steendieks Dubidoo</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>H2I1</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3096,37 +3171,38 @@
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Edwards, Susan</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>JP Zeppelin</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>H223</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Second Level Test 3</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Joan Williams at C)</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3140,37 +3216,38 @@
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3184,37 +3261,38 @@
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3228,37 +3306,38 @@
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Kuhn, Malcolm</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Moon</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>H2UC</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>USDF Introductory Test C</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -3272,37 +3351,38 @@
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -3316,37 +3396,38 @@
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Gillman, Chynna</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Padme Zarma TF</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>213</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>First Level Test 3</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -3360,37 +3441,38 @@
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Hamilton, Susan</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Seraphina MS</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>2T3</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Training Level Test 3</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="J12" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -3404,37 +3486,38 @@
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr"/>
+      <c r="K13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -3448,37 +3531,38 @@
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>2I1</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare I</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="J14" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -3492,37 +3576,38 @@
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>233</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -3536,37 +3621,38 @@
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>2I2</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>FEI Intermediare II</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="J16" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Susan Mandas at C)</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -3580,37 +3666,38 @@
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Jackson, Jackie</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Bravada HSR</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>212</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>First Level Test 2</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>Hunter 2 (Jodi Lees at C)</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -3624,42 +3711,43 @@
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>2YH</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Young Horse Test of Choice (excl 7YO)</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Roberts Arena (Jodi Ely at C)</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr"/>
+      <c r="K18" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J18"/>
+  <autoFilter ref="A3:K18"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -3672,7 +3760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3680,11 +3768,13 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -3712,35 +3802,40 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Rider</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Horse</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Class #</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Class Name</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Arena #</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Arena Name</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -3758,37 +3853,38 @@
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Va Fiero</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>US4EF</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>USEF 4-Year-Old Test Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (Beverly Rogers at C; Agnes</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr"/>
+      <c r="K4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -3802,37 +3898,38 @@
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Franzsis HSR</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>DHGEF</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>USEF Developing Horse Grand Prix Test Markel/USEF Qualifying</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -3846,37 +3943,38 @@
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Matchmaker HSR</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3890,37 +3988,38 @@
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Edwards, Susan</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>JP Zeppelin</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>331</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 1</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t>Jumper Ring (Cheryl Holekamp at C)</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3934,37 +4033,38 @@
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Fiorenza HSR</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>333</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Third Level Test 3</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Hunter 1 (Christel Carlson at C)</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3978,37 +4078,38 @@
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Fleming-Kuhn, Kathryn</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Vholt</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>3PSG</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>FEI Prix St. Georges</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t>The Sanctuary (Gwen Ka'awaloa at C)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -4022,42 +4123,43 @@
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Wilton, Jordan</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Wild Card HSR</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>3FFS</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>FEI Freestyle Test of Choice</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="J10" s="3" t="inlineStr">
         <is>
           <t>R &amp; L Arena (B. Rogers at C; A. Billington at B)</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J10"/>
+  <autoFilter ref="A3:K10"/>
   <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>